<commit_message>
Remove commute and replace it with travel allowance (something the user can set in the settings page). New fee for weekend and holidays. New pricing engine, lessons stores all to be independent.
</commit_message>
<xml_diff>
--- a/Apolo/Assets/Excel/Template.xlsx
+++ b/Apolo/Assets/Excel/Template.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aruiz\source\repos\alexruizdev\Apolo\Apolo\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD3C5EA-C620-487D-86F3-B8E7E72EA1CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{495D0400-2F68-4BE7-97BA-F257A656FF75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
   </bookViews>
   <sheets>
-    <sheet name="Lessons" sheetId="1" r:id="rId1"/>
-    <sheet name="Invoices" sheetId="3" r:id="rId2"/>
+    <sheet name="Services" sheetId="8" r:id="rId1"/>
+    <sheet name="Payers" sheetId="7" r:id="rId2"/>
     <sheet name="Students" sheetId="4" r:id="rId3"/>
     <sheet name="Specifications" sheetId="5" r:id="rId4"/>
-    <sheet name="Payers" sheetId="7" r:id="rId5"/>
-    <sheet name="Services" sheetId="8" r:id="rId6"/>
+    <sheet name="Lessons" sheetId="1" r:id="rId5"/>
+    <sheet name="Invoices" sheetId="3" r:id="rId6"/>
     <sheet name="Profiles" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
   <si>
     <t>Lessons</t>
   </si>
@@ -123,9 +123,6 @@
   </si>
   <si>
     <t>Last name</t>
-  </si>
-  <si>
-    <t>Commute</t>
   </si>
   <si>
     <t>Specifications</t>
@@ -498,25 +495,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="84">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
+  <dxfs count="83">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1274,19 +1253,6 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -1407,46 +1373,277 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="3" tint="0.249977111117893"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="3" tint="0.249977111117893"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="6"/>
+          <bgColor theme="3" tint="0.24994659260841701"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="3" tint="0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="3" tint="0.249977111117893"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1566,219 +1763,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="3" tint="0.249977111117893"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="3" tint="0.249977111117893"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="6"/>
-          <bgColor theme="3" tint="0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="3" tint="0.249977111117893"/>
-        </left>
-        <right style="thin">
-          <color theme="3" tint="0.249977111117893"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1793,119 +1777,118 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:M6" insertRow="1" totalsRowShown="0" headerRowDxfId="83" dataDxfId="81" headerRowBorderDxfId="82" tableBorderDxfId="80">
-  <autoFilter ref="B5:M6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Student" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Service" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Is total price" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Price per student" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{0350D2EA-6D0F-4D17-BF70-FFF762F354F0}" name="Paid" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Attendance ID" dataDxfId="70"/>
-    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Student ID" dataDxfId="69"/>
-    <tableColumn id="13" xr3:uid="{05AE8549-9E32-42AB-9E0E-0BECB84ADE19}" name="Service ID" dataDxfId="68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="17">
+  <autoFilter ref="B5:D6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Invoices" displayName="Invoices" ref="B5:J6" insertRow="1" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
-  <autoFilter ref="B5:J6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="ID" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Name" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="61"/>
-    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer name" dataDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{3309E227-DE1E-43C5-A6B6-0EC92AFFC66E}" name="Student" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="59"/>
-    <tableColumn id="8" xr3:uid="{BC748279-6F8A-40CD-A73A-4EAEC24A6408}" name="Paid" dataDxfId="58"/>
-    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="57"/>
-    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="Line ID" dataDxfId="56"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28">
+  <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="25"/>
+    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="24"/>
+    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:G6" insertRow="1" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54" tableBorderDxfId="52">
-  <autoFilter ref="B5:G6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="6">
-    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="50"/>
-    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{4CABC10F-1A7F-4D86-B90B-E069B2B53969}" name="Commute" dataDxfId="48"/>
-    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="47"/>
-    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50">
+  <autoFilter ref="B5:F6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="5">
+    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="48"/>
+    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="47"/>
+    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:J6" insertRow="1" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" headerRowBorderDxfId="44" tableBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:J6" insertRow="1" totalsRowShown="0" headerRowDxfId="44" dataDxfId="42" headerRowBorderDxfId="43" tableBorderDxfId="41">
   <autoFilter ref="B5:J6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="39"/>
-    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="38"/>
-    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Online" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Service ID" dataDxfId="34"/>
-    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Student ID" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="38"/>
+    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="37"/>
+    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Online" dataDxfId="35"/>
+    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="34"/>
+    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Service ID" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Student ID" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="32" dataDxfId="30" headerRowBorderDxfId="31" tableBorderDxfId="29">
-  <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="26"/>
-    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="25"/>
-    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:M6" insertRow="1" totalsRowShown="0" headerRowDxfId="69" dataDxfId="67" headerRowBorderDxfId="68" tableBorderDxfId="66">
+  <autoFilter ref="B5:M6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Student" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Service" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Is total price" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Price per student" dataDxfId="59"/>
+    <tableColumn id="9" xr3:uid="{0350D2EA-6D0F-4D17-BF70-FFF762F354F0}" name="Paid" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="57"/>
+    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Attendance ID" dataDxfId="56"/>
+    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Student ID" dataDxfId="55"/>
+    <tableColumn id="13" xr3:uid="{05AE8549-9E32-42AB-9E0E-0BECB84ADE19}" name="Service ID" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18">
-  <autoFilter ref="B5:D6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Invoices" displayName="Invoices" ref="B5:J6" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="80" headerRowBorderDxfId="81" tableBorderDxfId="79">
+  <autoFilter ref="B5:J6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="ID" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Name" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer name" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{3309E227-DE1E-43C5-A6B6-0EC92AFFC66E}" name="Student" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="73"/>
+    <tableColumn id="8" xr3:uid="{BC748279-6F8A-40CD-A73A-4EAEC24A6408}" name="Paid" dataDxfId="72"/>
+    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="71"/>
+    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="Line ID" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10">
   <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="10"/>
-    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="9"/>
-    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="8"/>
-    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="7"/>
-    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="6"/>
-    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="5"/>
-    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="4"/>
-    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="3"/>
-    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="9"/>
+    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="7"/>
+    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="6"/>
+    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="5"/>
+    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="4"/>
+    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="3"/>
+    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="2"/>
+    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2227,6 +2210,350 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{349C6D3A-2581-4BC1-B198-043D81DE2DED}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="3" spans="1:5" ht="34.5" x14ac:dyDescent="0.45">
+      <c r="B3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="20"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="14"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD90C9EB-D6B8-4999-A37E-50FEE41AA263}">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="31.28515625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="60.28515625" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="3" spans="1:9" ht="34.5" x14ac:dyDescent="0.45">
+      <c r="B3" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:G3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E084E8AE-8C3A-446D-A929-54817F8C0DDF}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="34.5" x14ac:dyDescent="0.45">
+      <c r="B3" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59E97CD-50F3-44EA-A57D-8B54153DA60F}">
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="31.28515625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="3" spans="1:11" ht="34.5" x14ac:dyDescent="0.45">
+      <c r="B3" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:G3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{873B8EF7-62DE-4FCD-B8E3-460BB4D2C6F0}">
   <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -2361,7 +2688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEF98F2-4AC5-4AA1-85C9-545C3E11603A}">
   <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -2428,10 +2755,10 @@
         <v>10</v>
       </c>
       <c r="I5" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="15" t="s">
         <v>44</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>45</v>
       </c>
       <c r="K5" s="5"/>
     </row>
@@ -2459,358 +2786,6 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B3:G3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E084E8AE-8C3A-446D-A929-54817F8C0DDF}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
-    <col min="4" max="5" width="31.28515625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.7109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="3" spans="1:8" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="5"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:F3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59E97CD-50F3-44EA-A57D-8B54153DA60F}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
-    <col min="4" max="6" width="31.28515625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="23.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="3" spans="1:11" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="7"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:G3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD90C9EB-D6B8-4999-A37E-50FEE41AA263}">
-  <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
-    <col min="4" max="6" width="31.28515625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="23.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="60.28515625" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="5"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="14"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:G3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{349C6D3A-2581-4BC1-B198-043D81DE2DED}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="29.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="3" spans="1:5" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="20"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
-      <c r="B5" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B3:C3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2844,7 +2819,7 @@
     </row>
     <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -2871,34 +2846,34 @@
     <row r="5" spans="1:12" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="K5" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L5" s="5"/>
     </row>

</xml_diff>

<commit_message>
update export to excel delete archive
</commit_message>
<xml_diff>
--- a/Apolo/Assets/Excel/Template.xlsx
+++ b/Apolo/Assets/Excel/Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aruiz\source\repos\alexruizdev\Apolo\Apolo\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{495D0400-2F68-4BE7-97BA-F257A656FF75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C3D36C-BF27-4BF0-B46E-5AD1FE48286B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="6" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
   </bookViews>
   <sheets>
     <sheet name="Services" sheetId="8" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
   <si>
     <t>Lessons</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Online</t>
   </si>
   <si>
-    <t>Is total price</t>
-  </si>
-  <si>
     <t>Price per student</t>
   </si>
   <si>
@@ -180,6 +177,24 @@
   </si>
   <si>
     <t>Line ID</t>
+  </si>
+  <si>
+    <t>Weekend</t>
+  </si>
+  <si>
+    <t>Price / hour</t>
+  </si>
+  <si>
+    <t>Travel allowance</t>
+  </si>
+  <si>
+    <t>Weekend Fee</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Payer</t>
   </si>
 </sst>
 </file>
@@ -495,7 +510,168 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="83">
+  <dxfs count="88">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -780,6 +956,282 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF215C98"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFFFFFFF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="6"/>
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color theme="0"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color rgb="FF215C98"/>
@@ -892,38 +1344,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1029,48 +1449,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color theme="0"/>
-        </right>
-        <top/>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1253,38 +1631,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1433,43 +1779,6 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
@@ -1575,194 +1884,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FF215C98"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFFFFFFF"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="6"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </left>
-        <right style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1777,118 +1898,123 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:D6" insertRow="1" totalsRowShown="0" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="17">
-  <autoFilter ref="B5:D6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:E6" insertRow="1" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
+  <autoFilter ref="B5:E6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{F070E4D6-2A8B-4929-BF04-8530F193BF70}" name="Price" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="69"/>
+    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
   <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="25"/>
-    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="24"/>
-    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="61"/>
+    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="60"/>
+    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="56" dataDxfId="54" headerRowBorderDxfId="55" tableBorderDxfId="53">
   <autoFilter ref="B5:F6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="5">
-    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="48"/>
-    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="47"/>
-    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="51"/>
+    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="50"/>
+    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="49"/>
+    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:J6" insertRow="1" totalsRowShown="0" headerRowDxfId="44" dataDxfId="42" headerRowBorderDxfId="43" tableBorderDxfId="41">
-  <autoFilter ref="B5:J6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="38"/>
-    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="37"/>
-    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Online" dataDxfId="35"/>
-    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="34"/>
-    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Service ID" dataDxfId="33"/>
-    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Student ID" dataDxfId="32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="47" dataDxfId="45" headerRowBorderDxfId="46" tableBorderDxfId="44">
+  <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="41"/>
+    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="40"/>
+    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{4CB3842E-EB1D-45CA-9308-72C92977B251}" name="Online" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Weekend" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="37"/>
+    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Student ID" dataDxfId="36"/>
+    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Service ID" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:M6" insertRow="1" totalsRowShown="0" headerRowDxfId="69" dataDxfId="67" headerRowBorderDxfId="68" tableBorderDxfId="66">
-  <autoFilter ref="B5:M6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Student" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Service" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Is total price" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Price per student" dataDxfId="59"/>
-    <tableColumn id="9" xr3:uid="{0350D2EA-6D0F-4D17-BF70-FFF762F354F0}" name="Paid" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="57"/>
-    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Attendance ID" dataDxfId="56"/>
-    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Student ID" dataDxfId="55"/>
-    <tableColumn id="13" xr3:uid="{05AE8549-9E32-42AB-9E0E-0BECB84ADE19}" name="Service ID" dataDxfId="54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:Q6" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="85" headerRowBorderDxfId="86" tableBorderDxfId="84">
+  <autoFilter ref="B5:Q6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="16">
+    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="83"/>
+    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Student" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Service" dataDxfId="81"/>
+    <tableColumn id="18" xr3:uid="{856AA0AD-A9D2-4BC4-B64C-DD339BB060A4}" name="Price" dataDxfId="2"/>
+    <tableColumn id="19" xr3:uid="{F88A226A-165B-497E-A103-652D51B5F335}" name="Paid" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{F2CC646E-5F4F-4968-901D-FB64DDD94A6C}" name="Notes" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{6C9740E9-87C2-4CC6-9AAD-1D8340BBB1E2}" name="Price / hour" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="80"/>
+    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Price per student" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="79"/>
+    <tableColumn id="14" xr3:uid="{E380BC68-97E8-4AEA-AEA7-229CB9BBE907}" name="Travel allowance" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Weekend" dataDxfId="78"/>
+    <tableColumn id="15" xr3:uid="{E1686B38-6591-41DA-BC53-FA0A75D72633}" name="Weekend Fee" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="77"/>
+    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Attendance ID" dataDxfId="76"/>
+    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Student ID" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Invoices" displayName="Invoices" ref="B5:J6" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="80" headerRowBorderDxfId="81" tableBorderDxfId="79">
-  <autoFilter ref="B5:J6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="ID" dataDxfId="78"/>
-    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Name" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="76"/>
-    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer name" dataDxfId="75"/>
-    <tableColumn id="5" xr3:uid="{3309E227-DE1E-43C5-A6B6-0EC92AFFC66E}" name="Student" dataDxfId="74"/>
-    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="73"/>
-    <tableColumn id="8" xr3:uid="{BC748279-6F8A-40CD-A73A-4EAEC24A6408}" name="Paid" dataDxfId="72"/>
-    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="71"/>
-    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="Line ID" dataDxfId="70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Invoices" displayName="Invoices" ref="B5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31">
+  <autoFilter ref="B5:I6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="ID" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Name" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{BC748279-6F8A-40CD-A73A-4EAEC24A6408}" name="Paid" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="24"/>
+    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="Line ID" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
   <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="9"/>
-    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="8"/>
-    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="7"/>
-    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="5"/>
-    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="4"/>
-    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="3"/>
-    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="2"/>
-    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="18"/>
+    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="17"/>
+    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="16"/>
+    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="15"/>
+    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="14"/>
+    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="13"/>
+    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="12"/>
+    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="11"/>
+    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2211,7 +2337,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{349C6D3A-2581-4BC1-B198-043D81DE2DED}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
@@ -2221,41 +2347,45 @@
     <col min="5" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="1:5" ht="34.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" s="20"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D6" s="8"/>
+      <c r="E6" s="14"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
     </row>
@@ -2294,7 +2424,7 @@
     </row>
     <row r="3" spans="1:9" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -2314,25 +2444,25 @@
     <row r="5" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="D5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>32</v>
-      </c>
       <c r="H5" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" s="5"/>
     </row>
@@ -2371,7 +2501,7 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" style="2" customWidth="1"/>
     <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="31.28515625" style="2" customWidth="1"/>
     <col min="5" max="5" width="23.7109375" style="2" customWidth="1"/>
@@ -2388,7 +2518,7 @@
     </row>
     <row r="3" spans="1:7" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -2405,19 +2535,19 @@
     <row r="5" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="D5" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -2448,7 +2578,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59E97CD-50F3-44EA-A57D-8B54153DA60F}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
@@ -2459,10 +2589,11 @@
     <col min="8" max="8" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.85546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="2"/>
+    <col min="11" max="11" width="18.140625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2470,9 +2601,9 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="3" spans="1:11" ht="34.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -2480,7 +2611,7 @@
       <c r="F3" s="20"/>
       <c r="G3" s="20"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2491,13 +2622,13 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>4</v>
@@ -2506,23 +2637,26 @@
         <v>5</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="15" t="s">
-        <v>17</v>
+      <c r="H5" s="6" t="s">
+        <v>44</v>
       </c>
       <c r="I5" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K5" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="L5" s="5"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -2530,11 +2664,12 @@
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
-      <c r="H6" s="14"/>
+      <c r="H6" s="8"/>
       <c r="I6" s="14"/>
-      <c r="J6" s="7"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J6" s="14"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2555,7 +2690,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{873B8EF7-62DE-4FCD-B8E3-460BB4D2C6F0}">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
@@ -2564,18 +2699,20 @@
     <col min="4" max="4" width="31.28515625" style="2" customWidth="1"/>
     <col min="5" max="5" width="23.7109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="19" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" style="2" customWidth="1"/>
     <col min="8" max="8" width="16.140625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="21.28515625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="2"/>
+    <col min="9" max="9" width="15.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" style="2" customWidth="1"/>
     <col min="11" max="11" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="2"/>
+    <col min="15" max="15" width="9.140625" style="2"/>
+    <col min="16" max="16" width="14.140625" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2586,7 +2723,7 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="3" spans="1:14" ht="34.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:18" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
         <v>0</v>
       </c>
@@ -2596,7 +2733,7 @@
       <c r="F3" s="20"/>
       <c r="G3" s="21"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2611,7 +2748,7 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
     </row>
-    <row r="5" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
         <v>1</v>
@@ -2623,50 +2760,66 @@
         <v>4</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="J5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="K5" s="15" t="s">
+      <c r="L5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="O5" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="15" t="s">
+      <c r="P5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="15" t="s">
+      <c r="Q5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="N5" s="5"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="R5" s="5"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="7"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2690,22 +2843,22 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEF98F2-4AC5-4AA1-85C9-545C3E11603A}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="13" style="2" customWidth="1"/>
     <col min="3" max="3" width="26.140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="31.28515625" style="2" customWidth="1"/>
-    <col min="5" max="6" width="23.7109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19" style="2" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="2"/>
+    <col min="5" max="5" width="23.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19" style="2" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -2713,56 +2866,51 @@
       <c r="E1" s="16"/>
       <c r="F1" s="16"/>
       <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="5"/>
-    </row>
-    <row r="3" spans="1:11" ht="34.5" x14ac:dyDescent="0.45">
+      <c r="H1" s="5"/>
+    </row>
+    <row r="3" spans="1:10" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
       <c r="E3" s="20"/>
       <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="I5" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="J5" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -2772,20 +2920,18 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2819,7 +2965,7 @@
     </row>
     <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -2846,34 +2992,34 @@
     <row r="5" spans="1:12" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="K5" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L5" s="5"/>
     </row>

</xml_diff>

<commit_message>
Refactor invoicing. - Bills no can be invoice or ticket. - Lessons are simplified and contain only a student. - Attendance invoices have been removed. Instead lesson have reference to the bill. - Update lesson view. - Update template excel. - Simplify payer outstanding. - Fix tests. - New ticket PDF generation. - Remove find invoice (todo refactor to display invoices and edit them).
</commit_message>
<xml_diff>
--- a/Apolo/Assets/Excel/Template.xlsx
+++ b/Apolo/Assets/Excel/Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aruiz\source\repos\alexruizdev\Apolo\Apolo\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C3D36C-BF27-4BF0-B46E-5AD1FE48286B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8F3251-7064-40EF-BF90-3010A5B39B7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="6" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="5" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
   </bookViews>
   <sheets>
     <sheet name="Services" sheetId="8" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Students" sheetId="4" r:id="rId3"/>
     <sheet name="Specifications" sheetId="5" r:id="rId4"/>
     <sheet name="Lessons" sheetId="1" r:id="rId5"/>
-    <sheet name="Invoices" sheetId="3" r:id="rId6"/>
+    <sheet name="Bills" sheetId="3" r:id="rId6"/>
     <sheet name="Profiles" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="52">
   <si>
     <t>Lessons</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Online</t>
   </si>
   <si>
-    <t>Price per student</t>
-  </si>
-  <si>
     <t>Paid</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>Student ID</t>
   </si>
   <si>
-    <t>Attendance ID</t>
-  </si>
-  <si>
     <t>Lesson ID</t>
   </si>
   <si>
@@ -176,9 +170,6 @@
     <t>Payer ID</t>
   </si>
   <si>
-    <t>Line ID</t>
-  </si>
-  <si>
     <t>Weekend</t>
   </si>
   <si>
@@ -195,6 +186,21 @@
   </si>
   <si>
     <t>Payer</t>
+  </si>
+  <si>
+    <t>Final Price</t>
+  </si>
+  <si>
+    <t>Bill</t>
+  </si>
+  <si>
+    <t>Base price</t>
+  </si>
+  <si>
+    <t>Bill ID</t>
+  </si>
+  <si>
+    <t>Type</t>
   </si>
 </sst>
 </file>
@@ -238,7 +244,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,8 +269,14 @@
         <bgColor theme="6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor theme="6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -450,12 +462,29 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="5" tint="-0.249977111117893"/>
+        <color theme="8" tint="0.59999389629810485"/>
       </left>
-      <right/>
-      <top/>
+      <right style="thin">
+        <color theme="8" tint="0.59999389629810485"/>
+      </right>
+      <top style="thin">
+        <color theme="8" tint="0.59999389629810485"/>
+      </top>
       <bottom style="thin">
-        <color theme="5" tint="-0.249977111117893"/>
+        <color theme="8" tint="0.59999389629810485"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -463,7 +492,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -494,9 +523,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -506,6 +532,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,305 +564,76 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <name val="Century Gothic"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -874,9 +677,311 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <border>
+        <bottom style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="6"/>
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="3" tint="0.249977111117893"/>
+        </top>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="thin">
-          <color rgb="FF215C98"/>
+          <color theme="3" tint="0.249977111117893"/>
         </bottom>
       </border>
     </dxf>
@@ -897,7 +1002,6 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="6"/>
@@ -931,176 +1035,6 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FF215C98"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFFFFFFF"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="6"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </left>
-        <right style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -1153,6 +1087,24 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1631,6 +1583,24 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1719,114 +1689,180 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <border outline="0">
         <top style="thin">
-          <color theme="3" tint="0.249977111117893"/>
+          <color rgb="FF215C98"/>
         </top>
         <bottom style="thin">
-          <color theme="0"/>
+          <color rgb="FFFFFFFF"/>
         </bottom>
       </border>
     </dxf>
@@ -1841,11 +1877,12 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <border outline="0">
         <bottom style="thin">
-          <color theme="3" tint="0.249977111117893"/>
+          <color rgb="FF215C98"/>
         </bottom>
       </border>
     </dxf>
@@ -1866,6 +1903,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="6"/>
@@ -1898,123 +1936,123 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:E6" insertRow="1" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:E6" insertRow="1" totalsRowShown="0" headerRowDxfId="73" dataDxfId="71" headerRowBorderDxfId="72" tableBorderDxfId="70">
   <autoFilter ref="B5:E6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{F070E4D6-2A8B-4929-BF04-8530F193BF70}" name="Price" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{F070E4D6-2A8B-4929-BF04-8530F193BF70}" name="Price" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="67"/>
+    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="65" dataDxfId="63" headerRowBorderDxfId="64" tableBorderDxfId="62">
   <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="61"/>
-    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="60"/>
-    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="59"/>
+    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="58"/>
+    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="56"/>
+    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="56" dataDxfId="54" headerRowBorderDxfId="55" tableBorderDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="54" dataDxfId="52" headerRowBorderDxfId="53" tableBorderDxfId="51">
   <autoFilter ref="B5:F6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="5">
-    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="51"/>
-    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="50"/>
-    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="49"/>
-    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="49"/>
+    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="47"/>
+    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="47" dataDxfId="45" headerRowBorderDxfId="46" tableBorderDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="45" dataDxfId="43" headerRowBorderDxfId="44" tableBorderDxfId="42">
   <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="41"/>
-    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="40"/>
-    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{4CB3842E-EB1D-45CA-9308-72C92977B251}" name="Online" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Weekend" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="37"/>
-    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Student ID" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Service ID" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="39"/>
+    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="38"/>
+    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{4CB3842E-EB1D-45CA-9308-72C92977B251}" name="Online" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Weekend" dataDxfId="35"/>
+    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="34"/>
+    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Student ID" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Service ID" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:Q6" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="85" headerRowBorderDxfId="86" tableBorderDxfId="84">
-  <autoFilter ref="B5:Q6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="83"/>
-    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Student" dataDxfId="82"/>
-    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Service" dataDxfId="81"/>
-    <tableColumn id="18" xr3:uid="{856AA0AD-A9D2-4BC4-B64C-DD339BB060A4}" name="Price" dataDxfId="2"/>
-    <tableColumn id="19" xr3:uid="{F88A226A-165B-497E-A103-652D51B5F335}" name="Paid" dataDxfId="1"/>
-    <tableColumn id="20" xr3:uid="{F2CC646E-5F4F-4968-901D-FB64DDD94A6C}" name="Notes" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{6C9740E9-87C2-4CC6-9AAD-1D8340BBB1E2}" name="Price / hour" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Price per student" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="79"/>
-    <tableColumn id="14" xr3:uid="{E380BC68-97E8-4AEA-AEA7-229CB9BBE907}" name="Travel allowance" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Weekend" dataDxfId="78"/>
-    <tableColumn id="15" xr3:uid="{E1686B38-6591-41DA-BC53-FA0A75D72633}" name="Weekend Fee" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Attendance ID" dataDxfId="76"/>
-    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Student ID" dataDxfId="75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:R6" insertRow="1" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28">
+  <autoFilter ref="B5:R6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="17">
+    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Service" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Student" dataDxfId="25"/>
+    <tableColumn id="18" xr3:uid="{856AA0AD-A9D2-4BC4-B64C-DD339BB060A4}" name="Final Price" dataDxfId="24"/>
+    <tableColumn id="19" xr3:uid="{F88A226A-165B-497E-A103-652D51B5F335}" name="Paid" dataDxfId="23"/>
+    <tableColumn id="20" xr3:uid="{F2CC646E-5F4F-4968-901D-FB64DDD94A6C}" name="Notes" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{8F080EB1-2903-456C-965B-2C7056063FA0}" name="Bill" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{6C9740E9-87C2-4CC6-9AAD-1D8340BBB1E2}" name="Price / hour" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="20"/>
+    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Base price" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="18"/>
+    <tableColumn id="14" xr3:uid="{E380BC68-97E8-4AEA-AEA7-229CB9BBE907}" name="Travel allowance" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Weekend" dataDxfId="16"/>
+    <tableColumn id="15" xr3:uid="{E1686B38-6591-41DA-BC53-FA0A75D72633}" name="Weekend Fee" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Student ID" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Bill ID" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Invoices" displayName="Invoices" ref="B5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31">
-  <autoFilter ref="B5:I6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="ID" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Name" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{BC748279-6F8A-40CD-A73A-4EAEC24A6408}" name="Paid" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="24"/>
-    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="Line ID" dataDxfId="23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Invoices" displayName="Invoices" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
+  <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="Name" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Type" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="ID" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="85" headerRowBorderDxfId="86" tableBorderDxfId="84">
   <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="17"/>
-    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="16"/>
-    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="15"/>
-    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="14"/>
-    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="13"/>
-    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="12"/>
-    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="11"/>
-    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="83"/>
+    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="82"/>
+    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="81"/>
+    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="80"/>
+    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="79"/>
+    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="78"/>
+    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="77"/>
+    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="76"/>
+    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2352,10 +2390,10 @@
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="20"/>
+      <c r="B3" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="19"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
@@ -2368,13 +2406,13 @@
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F5" s="5"/>
     </row>
@@ -2423,14 +2461,14 @@
       <c r="G1" s="1"/>
     </row>
     <row r="3" spans="1:9" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
+      <c r="B3" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
@@ -2444,25 +2482,25 @@
     <row r="5" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>31</v>
-      </c>
       <c r="H5" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I5" s="5"/>
     </row>
@@ -2517,12 +2555,12 @@
       <c r="E1" s="1"/>
     </row>
     <row r="3" spans="1:7" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
+      <c r="B3" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
@@ -2535,19 +2573,19 @@
     <row r="5" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -2602,14 +2640,14 @@
       <c r="G1" s="1"/>
     </row>
     <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
+      <c r="B3" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
@@ -2628,7 +2666,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>4</v>
@@ -2637,22 +2675,22 @@
         <v>5</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L5" s="5"/>
     </row>
@@ -2690,7 +2728,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{873B8EF7-62DE-4FCD-B8E3-460BB4D2C6F0}">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
@@ -2709,10 +2747,12 @@
     <col min="14" max="14" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9.140625" style="2"/>
     <col min="16" max="16" width="14.140625" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="2"/>
+    <col min="17" max="17" width="9.140625" style="2"/>
+    <col min="18" max="18" width="15.42578125" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2723,17 +2763,17 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="3" spans="1:18" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
+    <row r="3" spans="1:19" ht="34.5" x14ac:dyDescent="0.45">
+      <c r="B3" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="21"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="20"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2747,60 +2787,64 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-    </row>
-    <row r="5" spans="1:18" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:19" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>4</v>
-      </c>
       <c r="E5" s="6" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="L5" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="M5" s="6" t="s">
+      <c r="M5" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="N5" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="O5" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="N5" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="O5" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="P5" s="15" t="s">
-        <v>14</v>
+      <c r="P5" s="21" t="s">
+        <v>13</v>
       </c>
       <c r="Q5" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="R5" s="5"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="R5" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="S5" s="5"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
@@ -2809,17 +2853,18 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="8"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="12"/>
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="7"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="14"/>
       <c r="Q6" s="7"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R6" s="7"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2869,13 +2914,13 @@
       <c r="H1" s="5"/>
     </row>
     <row r="3" spans="1:10" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="B3" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="H4" s="3"/>
@@ -2885,30 +2930,27 @@
     <row r="5" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="17" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>9</v>
+        <v>18</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" s="5"/>
+        <v>14</v>
+      </c>
+      <c r="I5" s="5"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
@@ -2919,7 +2961,6 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
@@ -2964,18 +3005,18 @@
       <c r="K1" s="1"/>
     </row>
     <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
-      <c r="B3" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
+      <c r="B3" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
@@ -2992,34 +3033,34 @@
     <row r="5" spans="1:12" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>41</v>
-      </c>
       <c r="K5" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="L5" s="5"/>
     </row>

</xml_diff>

<commit_message>
Final version of excel backup
</commit_message>
<xml_diff>
--- a/Apolo/Assets/Excel/Template.xlsx
+++ b/Apolo/Assets/Excel/Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aruiz\source\repos\alexruizdev\Apolo\Apolo\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC223A67-7189-4900-9389-1A63A2845F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B203FFE-5858-465E-9140-06F42791270F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="19440" windowHeight="14880" activeTab="5" xr2:uid="{AC1E564E-6DB8-4849-BF2A-83F157C7F386}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="55">
   <si>
     <t>Lessons</t>
   </si>
@@ -134,9 +134,6 @@
     <t>City</t>
   </si>
   <si>
-    <t>NIF/CIF</t>
-  </si>
-  <si>
     <t>Services</t>
   </si>
   <si>
@@ -201,6 +198,18 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <t>Tip</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Sequence</t>
+  </si>
+  <si>
+    <t>Tax Id</t>
   </si>
 </sst>
 </file>
@@ -492,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -538,11 +547,67 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="88">
+  <dxfs count="91">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Century Gothic"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1936,123 +2001,126 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:E6" insertRow="1" totalsRowShown="0" headerRowDxfId="76" dataDxfId="74" headerRowBorderDxfId="75" tableBorderDxfId="73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C0795F78-0156-4685-AF9B-C080EB165C86}" name="Services" displayName="Services" ref="B5:E6" insertRow="1" totalsRowShown="0" headerRowDxfId="79" dataDxfId="77" headerRowBorderDxfId="78" tableBorderDxfId="76">
   <autoFilter ref="B5:E6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{F070E4D6-2A8B-4929-BF04-8530F193BF70}" name="Price" dataDxfId="71"/>
-    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="70"/>
-    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="69"/>
+    <tableColumn id="1" xr3:uid="{0421A27A-273F-4193-83E8-232DCB727B04}" name="Name" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{F070E4D6-2A8B-4929-BF04-8530F193BF70}" name="Price" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{322E168C-94B6-4464-82B7-AE5BD1C86BBE}" name="Price / h" dataDxfId="73"/>
+    <tableColumn id="10" xr3:uid="{699229C5-F45C-42AE-B09B-A008CEFA4B73}" name="ID" dataDxfId="72"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="68" dataDxfId="66" headerRowBorderDxfId="67" tableBorderDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0A79F4B1-F900-45BC-9D44-285E808E7870}" name="Payers" displayName="Payers" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="71" dataDxfId="69" headerRowBorderDxfId="70" tableBorderDxfId="68">
   <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="62"/>
-    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="61"/>
-    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="NIF/CIF" dataDxfId="59"/>
-    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{5BA77401-135F-49A0-9018-51E3A0234CED}" name="First name" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{EDB180AC-1296-443F-B84C-4D4EE4AE073B}" name="Last name" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{DCE1ACAA-6DAD-4705-81EB-7DFA2DF001BC}" name="Address" dataDxfId="65"/>
+    <tableColumn id="14" xr3:uid="{5B929BF7-C179-40AD-A842-4DFB12038777}" name="Zip code" dataDxfId="64"/>
+    <tableColumn id="15" xr3:uid="{6D6E1C47-E3A4-4383-BEC9-B9EAA078358A}" name="City" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{932DDB97-98FA-4056-8148-3C1EBD8A6957}" name="Tax Id" dataDxfId="62"/>
+    <tableColumn id="10" xr3:uid="{E234FAE6-CB9B-4EA0-B055-27B95F566BDE}" name="ID" dataDxfId="61"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="57" dataDxfId="55" headerRowBorderDxfId="56" tableBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{921EB506-3A8A-4A0B-B4FB-962E1B230FC8}" name="Students" displayName="Students" ref="B5:F6" insertRow="1" totalsRowShown="0" headerRowDxfId="60" dataDxfId="58" headerRowBorderDxfId="59" tableBorderDxfId="57">
   <autoFilter ref="B5:F6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="5">
-    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="52"/>
-    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="51"/>
-    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="50"/>
-    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{D3B37E7D-9062-40D6-B2B2-0A50D2AF30D8}" name="First name" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{DA765E80-CB03-496C-AB85-04C12F7F6EA1}" name="Last name" dataDxfId="55"/>
+    <tableColumn id="14" xr3:uid="{59DCAFC2-89B1-4CB1-9CF4-2945D31AD0A7}" name="Payer name" dataDxfId="54"/>
+    <tableColumn id="10" xr3:uid="{1186A2E8-3B8B-4232-BAAC-F12E28103DE4}" name="Id" dataDxfId="53"/>
+    <tableColumn id="11" xr3:uid="{2C87B7EC-1CBC-4BF1-BC1B-A80BEE6DF561}" name="PayerId" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="48" dataDxfId="46" headerRowBorderDxfId="47" tableBorderDxfId="45">
-  <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="42"/>
-    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="41"/>
-    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{4CB3842E-EB1D-45CA-9308-72C92977B251}" name="Online" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Weekend" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="37"/>
-    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Student ID" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Service ID" dataDxfId="35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AD4BFF54-6050-4EA0-B5EE-4251BB923ED8}" name="Specifications" displayName="Specifications" ref="B5:L6" insertRow="1" totalsRowShown="0" headerRowDxfId="51" dataDxfId="49" headerRowBorderDxfId="50" tableBorderDxfId="48">
+  <autoFilter ref="B5:L6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{A984BEB5-CD0A-4CBC-8261-5202F875C894}" name="Name" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{E5D86B37-BC1B-421B-8F67-1924F653B36B}" name="Student name" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{4F31CB14-2A08-4670-A72E-704E0461B7C0}" name="Service" dataDxfId="45"/>
+    <tableColumn id="14" xr3:uid="{2046F612-0B54-4B4A-8FFD-EC5D6AB309E9}" name="Duration" dataDxfId="44"/>
+    <tableColumn id="15" xr3:uid="{3B56031F-69EE-48E1-914B-517D98BD2AF6}" name="Price" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{4CB3842E-EB1D-45CA-9308-72C92977B251}" name="Online" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{E7ED6501-C9FE-4D56-95A1-F6238FF1D18F}" name="Weekend" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{9253E908-3CAE-4F64-B5A8-B2F87F28BA64}" name="Usage" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{AC948A85-76D1-41F8-8643-7143CFC6B853}" name="ID" dataDxfId="40"/>
+    <tableColumn id="16" xr3:uid="{97831813-DA71-41F9-9C8D-B5BDF0ABEBAF}" name="Student ID" dataDxfId="39"/>
+    <tableColumn id="11" xr3:uid="{CF31A15E-2BAA-48FB-B0FE-4AE64ECEA47C}" name="Service ID" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:R6" insertRow="1" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31">
-  <autoFilter ref="B5:R6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Service" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Student" dataDxfId="28"/>
-    <tableColumn id="18" xr3:uid="{856AA0AD-A9D2-4BC4-B64C-DD339BB060A4}" name="Final Price" dataDxfId="27"/>
-    <tableColumn id="19" xr3:uid="{F88A226A-165B-497E-A103-652D51B5F335}" name="Paid" dataDxfId="26"/>
-    <tableColumn id="20" xr3:uid="{F2CC646E-5F4F-4968-901D-FB64DDD94A6C}" name="Notes" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{8F080EB1-2903-456C-965B-2C7056063FA0}" name="Bill" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{6C9740E9-87C2-4CC6-9AAD-1D8340BBB1E2}" name="Price / hour" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Base price" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{E380BC68-97E8-4AEA-AEA7-229CB9BBE907}" name="Travel allowance" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Weekend" dataDxfId="18"/>
-    <tableColumn id="15" xr3:uid="{E1686B38-6591-41DA-BC53-FA0A75D72633}" name="Weekend Fee" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Student ID" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Bill ID" dataDxfId="14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}" name="Lessons" displayName="Lessons" ref="B5:S6" insertRow="1" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34">
+  <autoFilter ref="B5:S6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="18">
+    <tableColumn id="1" xr3:uid="{C1CFA75B-DE21-4250-99D5-6D2B34197E9D}" name="Date" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{E13660C3-AD05-4CF3-9631-AE40C9F89101}" name="Service" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{18BEE297-19DF-4B3B-B4FD-CFAE8F7A6949}" name="Student" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{856AA0AD-A9D2-4BC4-B64C-DD339BB060A4}" name="Final Price" dataDxfId="30"/>
+    <tableColumn id="19" xr3:uid="{F88A226A-165B-497E-A103-652D51B5F335}" name="Paid" dataDxfId="29"/>
+    <tableColumn id="20" xr3:uid="{F2CC646E-5F4F-4968-901D-FB64DDD94A6C}" name="Notes" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{8F080EB1-2903-456C-965B-2C7056063FA0}" name="Bill" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{6C9740E9-87C2-4CC6-9AAD-1D8340BBB1E2}" name="Price / hour" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{6CA1B731-8C2F-4DA6-B472-EE33DF6113CD}" name="Duration (min)" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{7A134DA8-4763-4978-90B3-711AAD8B520E}" name="Base price" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{7DCD903B-2C97-4AD2-B1F7-E4B6242A2CC8}" name="Online" dataDxfId="23"/>
+    <tableColumn id="14" xr3:uid="{E380BC68-97E8-4AEA-AEA7-229CB9BBE907}" name="Travel allowance" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{96F08C18-13F5-448F-99C8-A2B2DE97A9B4}" name="Weekend" dataDxfId="21"/>
+    <tableColumn id="15" xr3:uid="{E1686B38-6591-41DA-BC53-FA0A75D72633}" name="Weekend Fee" dataDxfId="20"/>
+    <tableColumn id="13" xr3:uid="{FD6DAC84-1316-4CAE-AA51-82ADB0D93933}" name="Tip" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{08B3198D-C1DC-4D8E-A4DE-7250D3A7C710}" name="Lesson ID" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{D13F67C3-A32E-454C-AE4D-C716888F27CB}" name="Student ID" dataDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{9B183B96-B338-4F28-AD14-AC6E651B6858}" name="Bill ID" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Bills" displayName="Bills" ref="B5:H6" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="85" headerRowBorderDxfId="86" tableBorderDxfId="84">
-  <autoFilter ref="B5:H6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="Name" dataDxfId="83"/>
-    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Type" dataDxfId="82"/>
-    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer" dataDxfId="80"/>
-    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="79"/>
-    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="78"/>
-    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="ID" dataDxfId="77"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C992FC1D-929F-4FCC-8034-BD1DE7AB4724}" name="Bills" displayName="Bills" ref="B5:I6" insertRow="1" totalsRowShown="0" headerRowDxfId="90" dataDxfId="88" headerRowBorderDxfId="89" tableBorderDxfId="87">
+  <autoFilter ref="B5:I6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{C69805C5-2DE6-4F5E-8595-BD91192122FB}" name="Name" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{31887EF0-F959-496C-8E82-BFC9313A5BD4}" name="Type" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{BD335C6E-9933-48E1-94D0-D0E510EFF5FB}" name="Created UTC" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{899EB7AE-2A40-41FC-80B1-65CB3A3ADF6E}" name="Payer" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{BB6B6371-F4F3-4ED2-B36B-8B9F19FEC62D}" name="Total" dataDxfId="82"/>
+    <tableColumn id="12" xr3:uid="{8DFC1E1F-49ED-490A-A022-750D97F2DB5E}" name="Payer ID" dataDxfId="81"/>
+    <tableColumn id="13" xr3:uid="{B0BEC736-D1AC-4A3A-A050-D3DA3F256C81}" name="ID" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{D6452AA6-9AAA-4EB7-9676-1AB575F8BFA3}" name="Sequence" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A2CA2C87-2B1E-47CC-B98B-F6DB30254282}" name="Profiles" displayName="Profiles" ref="B5:K6" insertRow="1" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13">
   <autoFilter ref="B5:K6" xr:uid="{03081AB8-5B53-403B-BC5F-49AB53C274F2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="9"/>
-    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="8"/>
-    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="7"/>
-    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="5"/>
-    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="4"/>
-    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="3"/>
-    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="2"/>
-    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{2F7003BC-BC4F-49D1-8191-9B7B77A95DAD}" name="Full name" dataDxfId="12"/>
+    <tableColumn id="17" xr3:uid="{1ED8C0D8-B8BF-4CB8-BF2A-11954C2F7E1C}" name="Zip code" dataDxfId="11"/>
+    <tableColumn id="20" xr3:uid="{7DBD046D-D51C-4C4F-8604-D6DEC2103E43}" name="City" dataDxfId="10"/>
+    <tableColumn id="19" xr3:uid="{7D393146-6466-4F51-87B6-10B7C5614A6A}" name="Phone" dataDxfId="9"/>
+    <tableColumn id="18" xr3:uid="{C771F655-E405-4BB5-AD39-3D5A94E1BBE0}" name="CIF/NIF" dataDxfId="8"/>
+    <tableColumn id="23" xr3:uid="{0F800687-A552-4911-A84F-66F27E40B2E9}" name="Email" dataDxfId="7"/>
+    <tableColumn id="22" xr3:uid="{2B05B060-5CA2-4293-8190-C4310A9D436E}" name="Bank name" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{7D5301B1-5635-4EF9-88C0-B2D2B15286FD}" name="Bank account" dataDxfId="5"/>
+    <tableColumn id="24" xr3:uid="{9790EA57-CF62-4EF2-ACAE-3D1545D8BFD5}" name="IVA" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{FAC1AFDA-6CB4-4B8D-A36E-7D10AC1588CA}" name="Address" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2391,7 +2459,7 @@
     </row>
     <row r="3" spans="1:6" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C3" s="21"/>
     </row>
@@ -2409,7 +2477,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>14</v>
@@ -2497,7 +2565,7 @@
         <v>28</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>14</v>
@@ -2616,7 +2684,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59E97CD-50F3-44EA-A57D-8B54153DA60F}">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
@@ -2625,13 +2693,13 @@
     <col min="4" max="6" width="31.28515625" style="2" customWidth="1"/>
     <col min="7" max="7" width="23.7109375" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="2"/>
+    <col min="9" max="10" width="12.85546875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2639,7 +2707,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="20" t="s">
         <v>23</v>
       </c>
@@ -2649,7 +2717,7 @@
       <c r="F3" s="21"/>
       <c r="G3" s="21"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2659,8 +2727,9 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:12" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
         <v>2</v>
@@ -2681,20 +2750,23 @@
         <v>7</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I5" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="K5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="L5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="5"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5" s="5"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -2703,11 +2775,12 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
-      <c r="I6" s="14"/>
+      <c r="I6" s="8"/>
       <c r="J6" s="14"/>
-      <c r="K6" s="7"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K6" s="14"/>
+      <c r="L6" s="7"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2728,7 +2801,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{873B8EF7-62DE-4FCD-B8E3-460BB4D2C6F0}">
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="2" customWidth="1"/>
@@ -2745,14 +2818,14 @@
     <col min="12" max="12" width="14.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="2"/>
-    <col min="16" max="16" width="14.140625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="2"/>
-    <col min="18" max="18" width="15.42578125" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="2"/>
+    <col min="15" max="16" width="9.140625" style="2"/>
+    <col min="17" max="17" width="14.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" style="2"/>
+    <col min="19" max="19" width="15.42578125" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2763,7 +2836,7 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="3" spans="1:19" ht="34.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:20" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="20" t="s">
         <v>0</v>
       </c>
@@ -2773,7 +2846,7 @@
       <c r="F3" s="21"/>
       <c r="G3" s="22"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -2788,8 +2861,9 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
-    </row>
-    <row r="5" spans="1:19" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="3"/>
+    </row>
+    <row r="5" spans="1:20" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
         <v>1</v>
@@ -2801,50 +2875,53 @@
         <v>3</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J5" s="19" t="s">
         <v>6</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L5" s="19" t="s">
         <v>7</v>
       </c>
       <c r="M5" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="N5" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="O5" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="N5" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="O5" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="P5" s="18" t="s">
+      <c r="P5" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="Q5" s="15" t="s">
+      <c r="R5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="R5" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="S5" s="5"/>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="T5" s="5"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="9"/>
       <c r="C6" s="10"/>
@@ -2860,11 +2937,12 @@
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="7"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="14"/>
       <c r="R6" s="7"/>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S6" s="7"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -2933,24 +3011,26 @@
         <v>2</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D5" s="17" t="s">
         <v>15</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>18</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="5"/>
+      <c r="I5" s="15" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
@@ -2961,6 +3041,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
+      <c r="I6" s="25"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B7" s="7"/>
@@ -3006,7 +3087,7 @@
     </row>
     <row r="3" spans="1:12" ht="34.5" x14ac:dyDescent="0.45">
       <c r="B3" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" s="21"/>
       <c r="D3" s="21"/>
@@ -3033,7 +3114,7 @@
     <row r="5" spans="1:12" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>27</v>
@@ -3042,22 +3123,22 @@
         <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="K5" s="6" t="s">
         <v>26</v>

</xml_diff>